<commit_message>
fix(task-040): localize reviewer workbooks to Chinese
</commit_message>
<xml_diff>
--- a/docs/qa/TASK-040/reviewer-r1-blind-review.xlsx
+++ b/docs/qa/TASK-040/reviewer-r1-blind-review.xlsx
@@ -4,486 +4,489 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Review" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Instructions" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Metadata" state="visible" r:id="rId6"/>
+    <sheet sheetId="1" name="评审" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="说明" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="元数据" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2214" uniqueCount="367">
-  <si>
-    <t>Row</t>
-  </si>
-  <si>
-    <t>Blind Item ID</t>
-  </si>
-  <si>
-    <t>Scenario</t>
-  </si>
-  <si>
-    <t>Traveler Intent</t>
-  </si>
-  <si>
-    <t>POI A</t>
-  </si>
-  <si>
-    <t>A Prefecture</t>
-  </si>
-  <si>
-    <t>A Region</t>
-  </si>
-  <si>
-    <t>A Category</t>
-  </si>
-  <si>
-    <t>A Source 1</t>
-  </si>
-  <si>
-    <t>A Source 2</t>
-  </si>
-  <si>
-    <t>POI B</t>
-  </si>
-  <si>
-    <t>B Prefecture</t>
-  </si>
-  <si>
-    <t>B Region</t>
-  </si>
-  <si>
-    <t>B Category</t>
-  </si>
-  <si>
-    <t>B Source 1</t>
-  </si>
-  <si>
-    <t>B Source 2</t>
-  </si>
-  <si>
-    <t>Choice</t>
-  </si>
-  <si>
-    <t>Confidence</t>
-  </si>
-  <si>
-    <t>Note</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2216" uniqueCount="370">
+  <si>
+    <t>序号</t>
+  </si>
+  <si>
+    <t>盲审题目 ID</t>
+  </si>
+  <si>
+    <t>旅行场景</t>
+  </si>
+  <si>
+    <t>旅客需求</t>
+  </si>
+  <si>
+    <t>景点 A</t>
+  </si>
+  <si>
+    <t>A 所在都道府县</t>
+  </si>
+  <si>
+    <t>A 所在地区</t>
+  </si>
+  <si>
+    <t>A 类型</t>
+  </si>
+  <si>
+    <t>A 来源 1</t>
+  </si>
+  <si>
+    <t>A 来源 2</t>
+  </si>
+  <si>
+    <t>景点 B</t>
+  </si>
+  <si>
+    <t>B 所在都道府县</t>
+  </si>
+  <si>
+    <t>B 所在地区</t>
+  </si>
+  <si>
+    <t>B 类型</t>
+  </si>
+  <si>
+    <t>B 来源 1</t>
+  </si>
+  <si>
+    <t>B 来源 2</t>
+  </si>
+  <si>
+    <t>选择</t>
+  </si>
+  <si>
+    <t>置信度</t>
+  </si>
+  <si>
+    <t>备注</t>
   </si>
   <si>
     <t>R1-1786003A6C46</t>
   </si>
   <si>
-    <t>Shopping and city traveler</t>
-  </si>
-  <si>
-    <t>A traveler prefers shopping, lively neighborhoods, and contemporary city experiences.</t>
-  </si>
-  <si>
-    <t>Yakushima</t>
-  </si>
-  <si>
-    <t>Kagoshima</t>
-  </si>
-  <si>
-    <t>Kyushu</t>
-  </si>
-  <si>
-    <t>Natural place</t>
-  </si>
-  <si>
-    <t>Source 1</t>
-  </si>
-  <si>
-    <t>Source 2</t>
-  </si>
-  <si>
-    <t>Amanoiwato Shrine</t>
-  </si>
-  <si>
-    <t>Miyazaki</t>
-  </si>
-  <si>
-    <t>Shrine or religious site</t>
+    <t>购物与都市体验</t>
+  </si>
+  <si>
+    <t>喜欢购物、热闹街区与现代都市体验。</t>
+  </si>
+  <si>
+    <t>屋久岛</t>
+  </si>
+  <si>
+    <t>鹿儿岛县</t>
+  </si>
+  <si>
+    <t>九州</t>
+  </si>
+  <si>
+    <t>自然景点</t>
+  </si>
+  <si>
+    <t>来源 1</t>
+  </si>
+  <si>
+    <t>来源 2</t>
+  </si>
+  <si>
+    <t>天岩户神社</t>
+  </si>
+  <si>
+    <t>宫崎县</t>
+  </si>
+  <si>
+    <t>神社或宗教场所</t>
   </si>
   <si>
     <t>R1-0FD7581CFCF2</t>
   </si>
   <si>
-    <t>Hidden and local explorer</t>
-  </si>
-  <si>
-    <t>A repeat visitor prefers locally distinctive places away from the most obvious headline sights.</t>
-  </si>
-  <si>
-    <t>Hirosaki Castle</t>
-  </si>
-  <si>
-    <t>Aomori</t>
-  </si>
-  <si>
-    <t>Tohoku</t>
-  </si>
-  <si>
-    <t>Park</t>
-  </si>
-  <si>
-    <t>Nijō Castle</t>
-  </si>
-  <si>
-    <t>Kyoto</t>
-  </si>
-  <si>
-    <t>Kansai</t>
-  </si>
-  <si>
-    <t>Garden</t>
+    <t>在地小众探索</t>
+  </si>
+  <si>
+    <t>曾多次访问日本，希望探索具有地方特色、避开热门地标的地点。</t>
+  </si>
+  <si>
+    <t>弘前城</t>
+  </si>
+  <si>
+    <t>青森县</t>
+  </si>
+  <si>
+    <t>东北</t>
+  </si>
+  <si>
+    <t>公园</t>
+  </si>
+  <si>
+    <t>二条城</t>
+  </si>
+  <si>
+    <t>京都府</t>
+  </si>
+  <si>
+    <t>关西</t>
+  </si>
+  <si>
+    <t>庭园</t>
   </si>
   <si>
     <t>R1-FEE288DC7C8A</t>
   </si>
   <si>
-    <t>Moerenuma Park</t>
-  </si>
-  <si>
-    <t>Hokkaido</t>
-  </si>
-  <si>
-    <t>Art or cultural venue</t>
+    <t>莫埃来沼公园</t>
+  </si>
+  <si>
+    <t>北海道</t>
+  </si>
+  <si>
+    <t>艺术或文化场馆</t>
   </si>
   <si>
     <t>R1-391E1BC7595B</t>
   </si>
   <si>
-    <t>Food-focused traveler</t>
-  </si>
-  <si>
-    <t>A traveler wants food culture and local eating experiences to lead the day.</t>
-  </si>
-  <si>
-    <t>Osaka Aquarium Kaiyukan</t>
-  </si>
-  <si>
-    <t>Osaka</t>
-  </si>
-  <si>
-    <t>Entertainment venue</t>
-  </si>
-  <si>
-    <t>Odori Park</t>
+    <t>美食主题</t>
+  </si>
+  <si>
+    <t>希望以饮食文化和当地美食体验为行程核心。</t>
+  </si>
+  <si>
+    <t>海游馆</t>
+  </si>
+  <si>
+    <t>大阪府</t>
+  </si>
+  <si>
+    <t>娱乐设施</t>
+  </si>
+  <si>
+    <t>大通公园</t>
   </si>
   <si>
     <t>R1-24E24A9223E6</t>
   </si>
   <si>
-    <t>Relaxed and rest-oriented traveler</t>
-  </si>
-  <si>
-    <t>A traveler wants a calm, restorative day with a relaxed pace.</t>
-  </si>
-  <si>
-    <t>Kōchi Castle</t>
-  </si>
-  <si>
-    <t>Kochi</t>
-  </si>
-  <si>
-    <t>Shikoku</t>
-  </si>
-  <si>
-    <t>Historic place</t>
-  </si>
-  <si>
-    <t>Ghibli Museum</t>
-  </si>
-  <si>
-    <t>Tokyo</t>
-  </si>
-  <si>
-    <t>Kanto</t>
-  </si>
-  <si>
-    <t>Museum</t>
+    <t>轻松疗愈</t>
+  </si>
+  <si>
+    <t>希望以舒缓节奏度过平静、放松的一天。</t>
+  </si>
+  <si>
+    <t>高知城</t>
+  </si>
+  <si>
+    <t>高知县</t>
+  </si>
+  <si>
+    <t>四国</t>
+  </si>
+  <si>
+    <t>历史景点</t>
+  </si>
+  <si>
+    <t>三鹰之森吉卜力美术馆</t>
+  </si>
+  <si>
+    <t>东京都</t>
+  </si>
+  <si>
+    <t>关东</t>
+  </si>
+  <si>
+    <t>博物馆</t>
   </si>
   <si>
     <t>R1-FDDCE7E12452</t>
   </si>
   <si>
-    <t>Low crowd and queue tolerance</t>
-  </si>
-  <si>
-    <t>A traveler has low tolerance for crowds and long queues.</t>
-  </si>
-  <si>
-    <t>Kiyomizu-dera</t>
-  </si>
-  <si>
-    <t>Temple or religious site</t>
-  </si>
-  <si>
-    <t>Sensō-ji</t>
+    <t>避开拥挤</t>
+  </si>
+  <si>
+    <t>对拥挤人群和长时间排队的承受能力较低。</t>
+  </si>
+  <si>
+    <t>清水寺</t>
+  </si>
+  <si>
+    <t>寺庙或宗教场所</t>
+  </si>
+  <si>
+    <t>浅草寺</t>
   </si>
   <si>
     <t>R1-4BACF3D4D91A</t>
   </si>
   <si>
-    <t>Nikkō Tōshō-gū</t>
-  </si>
-  <si>
-    <t>Tochigi</t>
-  </si>
-  <si>
-    <t>Nagasaki Peace Park</t>
-  </si>
-  <si>
-    <t>Nagasaki</t>
+    <t>日光东照宫</t>
+  </si>
+  <si>
+    <t>栃木县</t>
+  </si>
+  <si>
+    <t>长崎和平公园</t>
+  </si>
+  <si>
+    <t>长崎县</t>
   </si>
   <si>
     <t>R1-96C4FB315928</t>
   </si>
   <si>
-    <t>Iya Valley</t>
-  </si>
-  <si>
-    <t>Tokushima</t>
-  </si>
-  <si>
-    <t>Tōdai-ji</t>
-  </si>
-  <si>
-    <t>Nara</t>
+    <t>祖谷溪</t>
+  </si>
+  <si>
+    <t>德岛县</t>
+  </si>
+  <si>
+    <t>东大寺</t>
+  </si>
+  <si>
+    <t>奈良县</t>
   </si>
   <si>
     <t>R1-CF777B2C937E</t>
   </si>
   <si>
-    <t>First-time iconic traveler</t>
-  </si>
-  <si>
-    <t>A first-time visitor wants a memorable, widely recognizable introduction to Japan.</t>
-  </si>
-  <si>
-    <t>Shibuya Crossing</t>
-  </si>
-  <si>
-    <t>Shopping area</t>
-  </si>
-  <si>
-    <t>Shiretoko National Park</t>
-  </si>
-  <si>
-    <t>Mountain or highland place</t>
+    <t>初次访日经典体验</t>
+  </si>
+  <si>
+    <t>首次前往日本，希望获得难忘且具有代表性的日本旅行体验。</t>
+  </si>
+  <si>
+    <t>涩谷十字路口</t>
+  </si>
+  <si>
+    <t>购物区域</t>
+  </si>
+  <si>
+    <t>知床国立公园</t>
+  </si>
+  <si>
+    <t>山岳或高原</t>
   </si>
   <si>
     <t>R1-4D09187083BF</t>
   </si>
   <si>
-    <t>Art and educational traveler</t>
-  </si>
-  <si>
-    <t>A traveler prioritizes art, museums, and educational cultural experiences.</t>
-  </si>
-  <si>
-    <t>Arashiyama</t>
-  </si>
-  <si>
-    <t>Matsumoto Castle</t>
-  </si>
-  <si>
-    <t>Nagano</t>
-  </si>
-  <si>
-    <t>Chubu</t>
+    <t>艺术与文化学习</t>
+  </si>
+  <si>
+    <t>重视艺术、博物馆与具有学习价值的文化体验。</t>
+  </si>
+  <si>
+    <t>岚山</t>
+  </si>
+  <si>
+    <t>松本城</t>
+  </si>
+  <si>
+    <t>长野县</t>
+  </si>
+  <si>
+    <t>中部</t>
   </si>
   <si>
     <t>R1-B0AC9845DA08</t>
   </si>
   <si>
-    <t>Tsurugaoka Hachimangū</t>
-  </si>
-  <si>
-    <t>Kanagawa</t>
+    <t>鹤冈八幡宫</t>
+  </si>
+  <si>
+    <t>神奈川县</t>
   </si>
   <si>
     <t>R1-87D77AD54B7A</t>
   </si>
   <si>
-    <t>Low walking and physical tolerance</t>
-  </si>
-  <si>
-    <t>A traveler has low tolerance for prolonged walking or physical effort.</t>
+    <t>少步行需求</t>
+  </si>
+  <si>
+    <t>对长时间步行或体力消耗的承受能力较低。</t>
   </si>
   <si>
     <t>R1-829228667766</t>
   </si>
   <si>
-    <t>Matsushima</t>
-  </si>
-  <si>
-    <t>Miyagi</t>
-  </si>
-  <si>
-    <t>Hiroshima Peace Memorial Museum</t>
-  </si>
-  <si>
-    <t>Hiroshima</t>
-  </si>
-  <si>
-    <t>Chugoku</t>
+    <t>松岛</t>
+  </si>
+  <si>
+    <t>宫城县</t>
+  </si>
+  <si>
+    <t>广岛和平纪念资料馆</t>
+  </si>
+  <si>
+    <t>广岛县</t>
+  </si>
+  <si>
+    <t>中国地区</t>
   </si>
   <si>
     <t>R1-4AF65E761A63</t>
   </si>
   <si>
-    <t>Photography and scenery</t>
-  </si>
-  <si>
-    <t>A traveler prioritizes rewarding photography opportunities and attractive scenery.</t>
-  </si>
-  <si>
-    <t>Zuihōden</t>
+    <t>摄影与风景</t>
+  </si>
+  <si>
+    <t>重视摄影机会和优美景观。</t>
+  </si>
+  <si>
+    <t>瑞凤殿</t>
   </si>
   <si>
     <t>R1-B7CA590C0145</t>
   </si>
   <si>
-    <t>Nature traveler</t>
-  </si>
-  <si>
-    <t>A traveler wants nature, landscapes, parks, or outdoor exploration.</t>
-  </si>
-  <si>
-    <t>Sannai-Maruyama Site</t>
-  </si>
-  <si>
-    <t>Dōtonbori</t>
-  </si>
-  <si>
-    <t>Food-related place</t>
+    <t>自然旅行</t>
+  </si>
+  <si>
+    <t>希望探索自然、山水、公园或户外景观。</t>
+  </si>
+  <si>
+    <t>三内丸山遗址</t>
+  </si>
+  <si>
+    <t>道顿堀</t>
+  </si>
+  <si>
+    <t>美食相关地点</t>
   </si>
   <si>
     <t>R1-53BAA66C5723</t>
   </si>
   <si>
-    <t>History and architecture</t>
-  </si>
-  <si>
-    <t>A traveler is especially interested in history, heritage, and architecture.</t>
-  </si>
-  <si>
-    <t>Osaka Castle</t>
-  </si>
-  <si>
-    <t>Rurikō-ji</t>
-  </si>
-  <si>
-    <t>Yamaguchi</t>
+    <t>历史与建筑</t>
+  </si>
+  <si>
+    <t>对历史、文化遗产与建筑尤其感兴趣。</t>
+  </si>
+  <si>
+    <t>大阪城</t>
+  </si>
+  <si>
+    <t>瑠璃光寺</t>
+  </si>
+  <si>
+    <t>山口县</t>
   </si>
   <si>
     <t>R1-F06590DAB9ED</t>
   </si>
   <si>
-    <t>Shitennō-ji</t>
-  </si>
-  <si>
-    <t>National Museum of Nature and Science</t>
+    <t>四天王寺</t>
+  </si>
+  <si>
+    <t>国立科学博物馆</t>
   </si>
   <si>
     <t>R1-3B4017057EE0</t>
   </si>
   <si>
-    <t>Mount Aso</t>
-  </si>
-  <si>
-    <t>Kumamoto</t>
+    <t>阿苏山</t>
+  </si>
+  <si>
+    <t>熊本县</t>
   </si>
   <si>
     <t>R1-558C8E9BBBC2</t>
   </si>
   <si>
-    <t>Lake Kawaguchi</t>
-  </si>
-  <si>
-    <t>Yamanashi</t>
-  </si>
-  <si>
-    <t>Scenic viewpoint</t>
-  </si>
-  <si>
-    <t>Toyota Commemorative Museum of Industry and Technology</t>
-  </si>
-  <si>
-    <t>Aichi</t>
+    <t>河口湖</t>
+  </si>
+  <si>
+    <t>山梨县</t>
+  </si>
+  <si>
+    <t>景观眺望点</t>
+  </si>
+  <si>
+    <t>丰田产业技术纪念馆</t>
+  </si>
+  <si>
+    <t>爱知县</t>
   </si>
   <si>
     <t>R1-9A4BF7CC4A9D</t>
   </si>
   <si>
-    <t>Naoshima</t>
-  </si>
-  <si>
-    <t>Kagawa</t>
+    <t>直岛町</t>
+  </si>
+  <si>
+    <t>香川县</t>
   </si>
   <si>
     <t>R1-FC9E0A8A9EC2</t>
   </si>
   <si>
-    <t>Hakone Open-Air Museum</t>
+    <t>箱根雕刻森林美术馆</t>
   </si>
   <si>
     <t>R1-091D7DCC9E02</t>
   </si>
   <si>
-    <t>Sapporo Clock Tower</t>
+    <t>札幌市钟楼</t>
   </si>
   <si>
     <t>R1-179D248A434F</t>
   </si>
   <si>
-    <t>Ginzan Onsen</t>
-  </si>
-  <si>
-    <t>Yamagata</t>
+    <t>银山温泉</t>
+  </si>
+  <si>
+    <t>山形县</t>
   </si>
   <si>
     <t>R1-E172605EEFEB</t>
   </si>
   <si>
-    <t>Oirase River</t>
-  </si>
-  <si>
-    <t>Tottori Sand Dunes</t>
-  </si>
-  <si>
-    <t>Tottori</t>
+    <t>奥入濑川</t>
+  </si>
+  <si>
+    <t>鸟取砂丘</t>
+  </si>
+  <si>
+    <t>鸟取县</t>
   </si>
   <si>
     <t>R1-401E735EB49C</t>
   </si>
   <si>
-    <t>Family and interactive soft fit</t>
-  </si>
-  <si>
-    <t>A family group prefers engaging, interactive places with broad age appeal.</t>
-  </si>
-  <si>
-    <t>Okinawa World</t>
-  </si>
-  <si>
-    <t>Okinawa</t>
+    <t>亲子互动</t>
+  </si>
+  <si>
+    <t>家庭同行，希望选择互动性强、适合不同年龄段的地点。</t>
+  </si>
+  <si>
+    <t>冲绳世界文化王国·玉泉洞</t>
+  </si>
+  <si>
+    <t>冲绳县</t>
+  </si>
+  <si>
+    <t>冲绳</t>
   </si>
   <si>
     <t>R1-D91D8AEA3C52</t>
   </si>
   <si>
-    <t>Shirakawa, Gifu (village)</t>
-  </si>
-  <si>
-    <t>Gifu</t>
-  </si>
-  <si>
-    <t>Atsuta Shrine</t>
+    <t>白川村</t>
+  </si>
+  <si>
+    <t>岐阜县</t>
+  </si>
+  <si>
+    <t>热田神宫</t>
   </si>
   <si>
     <t>R1-696C64EEF45B</t>
@@ -492,7 +495,7 @@
     <t>R1-E7F3FC885478</t>
   </si>
   <si>
-    <t>Meiji Shrine</t>
+    <t>明治神宫</t>
   </si>
   <si>
     <t>R1-004B2EBF7D54</t>
@@ -501,7 +504,7 @@
     <t>R1-FAEB6B6DAAEF</t>
   </si>
   <si>
-    <t>Tokyo Skytree</t>
+    <t>东京晴空塔</t>
   </si>
   <si>
     <t>R1-FCDA1334EEC1</t>
@@ -510,73 +513,73 @@
     <t>R1-E64EDF60BDF8</t>
   </si>
   <si>
-    <t>Himeji Castle</t>
-  </si>
-  <si>
-    <t>Hyogo</t>
+    <t>姬路城</t>
+  </si>
+  <si>
+    <t>兵库县</t>
   </si>
   <si>
     <t>R1-8E012EAE6BE4</t>
   </si>
   <si>
-    <t>Dōgo Onsen</t>
-  </si>
-  <si>
-    <t>Ehime</t>
+    <t>道后温泉</t>
+  </si>
+  <si>
+    <t>爱媛县</t>
   </si>
   <si>
     <t>R1-8874BCA5A131</t>
   </si>
   <si>
-    <t>Yokohama Chinatown</t>
-  </si>
-  <si>
-    <t>Hiroshima Peace Memorial</t>
+    <t>横滨中华街</t>
+  </si>
+  <si>
+    <t>原子弹爆炸圆顶屋</t>
   </si>
   <si>
     <t>R1-9854C9562BD0</t>
   </si>
   <si>
-    <t>Nagoya Castle</t>
+    <t>名古屋城</t>
   </si>
   <si>
     <t>R1-D6B727F62340</t>
   </si>
   <si>
-    <t>Sumiyoshi-taisha</t>
-  </si>
-  <si>
-    <t>Adachi Museum of Art</t>
-  </si>
-  <si>
-    <t>Shimane</t>
+    <t>住吉大社</t>
+  </si>
+  <si>
+    <t>足立美术馆</t>
+  </si>
+  <si>
+    <t>岛根县</t>
   </si>
   <si>
     <t>R1-80F0B0C0F49B</t>
   </si>
   <si>
-    <t>Kōtoku-in</t>
-  </si>
-  <si>
-    <t>Mōtsū-ji</t>
-  </si>
-  <si>
-    <t>Iwate</t>
+    <t>高德院</t>
+  </si>
+  <si>
+    <t>毛越寺</t>
+  </si>
+  <si>
+    <t>岩手县</t>
   </si>
   <si>
     <t>R1-7D8C5A89907F</t>
   </si>
   <si>
-    <t>Matsuyama Castle (Iyo)</t>
+    <t>松山城</t>
   </si>
   <si>
     <t>R1-893056051C8C</t>
   </si>
   <si>
-    <t>Kumamoto Castle</t>
-  </si>
-  <si>
-    <t>Itsukushima Shrine</t>
+    <t>熊本城</t>
+  </si>
+  <si>
+    <t>严岛神社</t>
   </si>
   <si>
     <t>R1-CD7CD3BA193C</t>
@@ -588,7 +591,7 @@
     <t>R1-ECE437C5126D</t>
   </si>
   <si>
-    <t>Zenkō-ji</t>
+    <t>善光寺</t>
   </si>
   <si>
     <t>R1-0F3AA9E001D8</t>
@@ -600,22 +603,22 @@
     <t>R1-B64F192F4DA1</t>
   </si>
   <si>
-    <t>Asahiyama Zoo</t>
-  </si>
-  <si>
-    <t>Okinawa Churaumi Aquarium</t>
+    <t>旭川市旭山动物园</t>
+  </si>
+  <si>
+    <t>冲绳美丽海水族馆</t>
   </si>
   <si>
     <t>R1-AE58CE4200E0</t>
   </si>
   <si>
-    <t>Chūson-ji</t>
+    <t>中尊寺</t>
   </si>
   <si>
     <t>R1-DCD1C8CAEDF5</t>
   </si>
   <si>
-    <t>Takayama Jin'ya</t>
+    <t>高山阵屋</t>
   </si>
   <si>
     <t>R1-8B23B78DF9B8</t>
@@ -624,22 +627,22 @@
     <t>R1-67C9D53B64D8</t>
   </si>
   <si>
-    <t>Gion</t>
+    <t>祇园</t>
   </si>
   <si>
     <t>R1-D4233AC67EE4</t>
   </si>
   <si>
-    <t>Fushimi Inari-taisha</t>
+    <t>伏见稻荷大社</t>
   </si>
   <si>
     <t>R1-9289C482F1A9</t>
   </si>
   <si>
-    <t>Sapporo TV Tower</t>
-  </si>
-  <si>
-    <t>Fuji-Q Highland</t>
+    <t>札幌电视塔</t>
+  </si>
+  <si>
+    <t>富士急高原乐园</t>
   </si>
   <si>
     <t>R1-38B555374A6C</t>
@@ -648,10 +651,10 @@
     <t>R1-C06F7563CFB7</t>
   </si>
   <si>
-    <t>Ueno Park</t>
-  </si>
-  <si>
-    <t>Kyoto National Museum</t>
+    <t>上野公园</t>
+  </si>
+  <si>
+    <t>京都国立博物馆</t>
   </si>
   <si>
     <t>R1-E9469EBE4FDB</t>
@@ -660,10 +663,10 @@
     <t>R1-C6D3E17CEA22</t>
   </si>
   <si>
-    <t>Lake Towada</t>
-  </si>
-  <si>
-    <t>Ritsurin Garden</t>
+    <t>十和田湖</t>
+  </si>
+  <si>
+    <t>栗林公园</t>
   </si>
   <si>
     <t>R1-E8837C720AFB</t>
@@ -672,13 +675,13 @@
     <t>R1-7DBCF6763F59</t>
   </si>
   <si>
-    <t>Tokyo Tower</t>
+    <t>东京铁塔</t>
   </si>
   <si>
     <t>R1-5A5C69CE6380</t>
   </si>
   <si>
-    <t>Universal Studios Japan</t>
+    <t>日本环球影城</t>
   </si>
   <si>
     <t>R1-1E15F9397015</t>
@@ -690,10 +693,10 @@
     <t>R1-61664338894A</t>
   </si>
   <si>
-    <t>Tsukiji fish market</t>
-  </si>
-  <si>
-    <t>Market</t>
+    <t>筑地市场</t>
+  </si>
+  <si>
+    <t>市场</t>
   </si>
   <si>
     <t>R1-7218A006BDCA</t>
@@ -714,7 +717,7 @@
     <t>R1-FA945E0AD1B0</t>
   </si>
   <si>
-    <t>Okinawa Prefectural Museum</t>
+    <t>冲绳县立博物馆、美术馆</t>
   </si>
   <si>
     <t>R1-A8C19DFFAB4A</t>
@@ -723,10 +726,10 @@
     <t>R1-5B7655C528C8</t>
   </si>
   <si>
-    <t>Mount Fuji</t>
-  </si>
-  <si>
-    <t>Shizuoka</t>
+    <t>富士山</t>
+  </si>
+  <si>
+    <t>静冈县</t>
   </si>
   <si>
     <t>R1-3B7C4D2B3659</t>
@@ -735,16 +738,16 @@
     <t>R1-CD272B7FE0EB</t>
   </si>
   <si>
-    <t>Kōraku-en</t>
-  </si>
-  <si>
-    <t>Okayama</t>
+    <t>后乐园</t>
+  </si>
+  <si>
+    <t>冈山县</t>
   </si>
   <si>
     <t>R1-FC5FAD5FD6FD</t>
   </si>
   <si>
-    <t>Jigokudani Monkey Park</t>
+    <t>地狱谷野猿公苑</t>
   </si>
   <si>
     <t>R1-17E0EB55C248</t>
@@ -753,13 +756,13 @@
     <t>R1-8D18D50D1BDA</t>
   </si>
   <si>
-    <t>Naruto whirlpools</t>
+    <t>鸣门漩涡</t>
   </si>
   <si>
     <t>R1-D2222C04EE66</t>
   </si>
   <si>
-    <t>Sakurajima</t>
+    <t>樱岛</t>
   </si>
   <si>
     <t>R1-42F780213CE2</t>
@@ -777,16 +780,16 @@
     <t>R1-A9347BB53190</t>
   </si>
   <si>
-    <t>Huis Ten Bosch (theme park)</t>
+    <t>豪斯登堡</t>
   </si>
   <si>
     <t>R1-DE6943552F5D</t>
   </si>
   <si>
-    <t>Ise Shrine</t>
-  </si>
-  <si>
-    <t>Mie</t>
+    <t>伊势神宫</t>
+  </si>
+  <si>
+    <t>三重县</t>
   </si>
   <si>
     <t>R1-ECA39FB42859</t>
@@ -798,16 +801,16 @@
     <t>R1-17E1D60036D4</t>
   </si>
   <si>
-    <t>Tokyo Disneyland</t>
-  </si>
-  <si>
-    <t>Chiba</t>
+    <t>东京迪士尼乐园</t>
+  </si>
+  <si>
+    <t>千叶县</t>
   </si>
   <si>
     <t>R1-FF21FDB4BEA5</t>
   </si>
   <si>
-    <t>Yama-dera</t>
+    <t>立石寺</t>
   </si>
   <si>
     <t>R1-7C9050C78155</t>
@@ -822,7 +825,7 @@
     <t>R1-F77CCE692AFA</t>
   </si>
   <si>
-    <t>Cape Manzamo</t>
+    <t>万座毛</t>
   </si>
   <si>
     <t>R1-A831659FEAE8</t>
@@ -837,13 +840,13 @@
     <t>R1-AF2699E3550A</t>
   </si>
   <si>
-    <t>Nara Park</t>
+    <t>奈良公园</t>
   </si>
   <si>
     <t>R1-9229B0DDE6D4</t>
   </si>
   <si>
-    <t>Ōtsuka Museum of Art</t>
+    <t>大冢国际美术馆</t>
   </si>
   <si>
     <t>R1-C425659DDBA4</t>
@@ -858,7 +861,7 @@
     <t>R1-FCA44F0AC917</t>
   </si>
   <si>
-    <t>Izumo-taisha</t>
+    <t>出云大社</t>
   </si>
   <si>
     <t>R1-080FC1D9F87D</t>
@@ -870,7 +873,7 @@
     <t>R1-44894B05A1D4</t>
   </si>
   <si>
-    <t>Lake Mashū</t>
+    <t>摩周湖</t>
   </si>
   <si>
     <t>R1-10B96A27223E</t>
@@ -897,10 +900,10 @@
     <t>R1-4BEF5ACFEA04</t>
   </si>
   <si>
-    <t>Kusatsu Onsen</t>
-  </si>
-  <si>
-    <t>Gunma</t>
+    <t>草津温泉</t>
+  </si>
+  <si>
+    <t>群马县</t>
   </si>
   <si>
     <t>R1-CBFE77F0A930</t>
@@ -999,13 +1002,13 @@
     <t>R1-862F008B59D5</t>
   </si>
   <si>
-    <t>Kenroku-en</t>
-  </si>
-  <si>
-    <t>Ishikawa</t>
-  </si>
-  <si>
-    <t>Arima Onsen</t>
+    <t>兼六园</t>
+  </si>
+  <si>
+    <t>石川县</t>
+  </si>
+  <si>
+    <t>有马温泉</t>
   </si>
   <si>
     <t>R1-9181F39133C6</t>
@@ -1017,103 +1020,109 @@
     <t>R1-D01A6838460C</t>
   </si>
   <si>
-    <t>Reviewer Instructions</t>
-  </si>
-  <si>
-    <t>Guidance</t>
-  </si>
-  <si>
-    <t>Purpose</t>
-  </si>
-  <si>
-    <t>Judge which POI better fits the stated traveler scenario. Judge traveler fit, not your personal favorite.</t>
-  </si>
-  <si>
-    <t>Choose exactly one: A, B, TIE, or INSUFFICIENT_INFO.</t>
-  </si>
-  <si>
-    <t>Choose high, medium, or low for every answered row.</t>
-  </si>
-  <si>
-    <t>Independence</t>
-  </si>
-  <si>
-    <t>Work independently. Do not inspect TASK-038 files, restricted TASK-039 mapping files, scoring code, or another reviewer’s answers.</t>
-  </si>
-  <si>
-    <t>Evidence</t>
-  </si>
-  <si>
-    <t>Source links are neutral identity references. Open them only when identity or broad type is unclear.</t>
-  </si>
-  <si>
-    <t>Out of scope</t>
-  </si>
-  <si>
-    <t>Do not infer live opening hours, queues, weather, route feasibility, booking availability, or price inventory.</t>
-  </si>
-  <si>
-    <t>Insufficient information</t>
-  </si>
-  <si>
-    <t>Use INSUFFICIENT_INFO when the available information cannot support a responsible judgment.</t>
-  </si>
-  <si>
-    <t>Protected cells</t>
-  </si>
-  <si>
-    <t>Do not alter question, identity, or source cells. Only Choice, Confidence, and Note are intended for editing.</t>
-  </si>
-  <si>
-    <t>Privacy</t>
-  </si>
-  <si>
-    <t>Do not enter your name, contact details, or other personal information in Note.</t>
-  </si>
-  <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>reviewVersion</t>
+    <t>评审说明</t>
+  </si>
+  <si>
+    <t>操作指引</t>
+  </si>
+  <si>
+    <t>评审目标</t>
+  </si>
+  <si>
+    <t>判断哪个景点更符合给出的旅行场景。请判断旅客适配度，而不是选择您个人更喜欢的景点。</t>
+  </si>
+  <si>
+    <t>每题只能选择一项：A、B、平局或信息不足。</t>
+  </si>
+  <si>
+    <t>每道已作答题目都必须选择高、中或低。</t>
+  </si>
+  <si>
+    <t>独立性</t>
+  </si>
+  <si>
+    <t>请独立完成评审。不要查看 TASK-038 文件、受限的 TASK-039 映射文件、评分代码或其他评审员的答案。</t>
+  </si>
+  <si>
+    <t>来源</t>
+  </si>
+  <si>
+    <t>来源链接仅用于中立地确认景点身份。只有当景点身份或大类不明确时才需要打开。</t>
+  </si>
+  <si>
+    <t>评审范围外</t>
+  </si>
+  <si>
+    <t>不要推测实时营业时间、排队情况、天气、路线可行性、预约可用性或价格库存。</t>
+  </si>
+  <si>
+    <t>信息不足</t>
+  </si>
+  <si>
+    <t>当现有信息不足以支持可靠判断时，请选择“信息不足”。</t>
+  </si>
+  <si>
+    <t>受保护单元格</t>
+  </si>
+  <si>
+    <t>请勿修改题目、景点身份或来源单元格。只有“选择”“置信度”和“备注”允许填写。</t>
+  </si>
+  <si>
+    <t>隐私</t>
+  </si>
+  <si>
+    <t>请勿在备注中填写姓名、联系方式或其他个人信息。</t>
+  </si>
+  <si>
+    <t>字段</t>
+  </si>
+  <si>
+    <t>值</t>
+  </si>
+  <si>
+    <t>评审版本</t>
   </si>
   <si>
     <t>task-039-v1</t>
   </si>
   <si>
-    <t>reviewerCode</t>
+    <t>评审员代码</t>
   </si>
   <si>
     <t>R1</t>
   </si>
   <si>
-    <t>itemCount</t>
-  </si>
-  <si>
-    <t>sourcePackSha256</t>
+    <t>题目数量</t>
+  </si>
+  <si>
+    <t>源题包 SHA-256</t>
   </si>
   <si>
     <t>0ec82e3769b014fe42b78c76d2b5cd50d215344b84446fec20375ae83e7973b7</t>
   </si>
   <si>
-    <t>workbookSchemaVersion</t>
-  </si>
-  <si>
-    <t>task-040-xlsx-v1</t>
-  </si>
-  <si>
-    <t>protectedContentDigestAlgorithm</t>
+    <t>工作簿结构版本</t>
+  </si>
+  <si>
+    <t>task-040-xlsx-v2-zh-CN</t>
+  </si>
+  <si>
+    <t>受保护内容摘要算法</t>
   </si>
   <si>
     <t>SHA-256</t>
   </si>
   <si>
-    <t>protectedContentDigest</t>
-  </si>
-  <si>
-    <t>782f8b36c54cb4a66d8d123918235196e75ada1740e4d4a5415dfa25735d118b</t>
+    <t>受保护内容摘要</t>
+  </si>
+  <si>
+    <t>bfd32364745c9e6f6e6aa6464ec2e3c7864d843d9b34b784a8e04a4f31d01ab9</t>
+  </si>
+  <si>
+    <t>中文本地化目录 SHA-256</t>
+  </si>
+  <si>
+    <t>3598c6559a2ab5641091be1954c3e86b2ee62fb94b42c6a8a860de3b5e4a3b12</t>
   </si>
 </sst>
 </file>
@@ -2964,7 +2973,7 @@
         <v>152</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>51</v>
@@ -3002,7 +3011,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C27" s="10" t="s">
         <v>149</v>
@@ -3011,10 +3020,10 @@
         <v>150</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G27" s="10" t="s">
         <v>93</v>
@@ -3029,7 +3038,7 @@
         <v>27</v>
       </c>
       <c r="K27" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="L27" s="10" t="s">
         <v>133</v>
@@ -3055,7 +3064,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>65</v>
@@ -3064,10 +3073,10 @@
         <v>66</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>93</v>
@@ -3108,7 +3117,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C29" s="10" t="s">
         <v>107</v>
@@ -3135,7 +3144,7 @@
         <v>27</v>
       </c>
       <c r="K29" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L29" s="10" t="s">
         <v>61</v>
@@ -3161,7 +3170,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>117</v>
@@ -3214,7 +3223,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C31" s="10" t="s">
         <v>149</v>
@@ -3241,7 +3250,7 @@
         <v>27</v>
       </c>
       <c r="K31" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L31" s="10" t="s">
         <v>61</v>
@@ -3267,7 +3276,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>65</v>
@@ -3320,7 +3329,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C33" s="10" t="s">
         <v>32</v>
@@ -3329,10 +3338,10 @@
         <v>33</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G33" s="10" t="s">
         <v>40</v>
@@ -3373,7 +3382,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>88</v>
@@ -3400,10 +3409,10 @@
         <v>27</v>
       </c>
       <c r="K34" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M34" s="5" t="s">
         <v>58</v>
@@ -3426,7 +3435,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C35" s="10" t="s">
         <v>149</v>
@@ -3435,7 +3444,7 @@
         <v>150</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>96</v>
@@ -3453,7 +3462,7 @@
         <v>27</v>
       </c>
       <c r="K35" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L35" s="10" t="s">
         <v>104</v>
@@ -3479,7 +3488,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>20</v>
@@ -3488,7 +3497,7 @@
         <v>21</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F36" s="5" t="s">
         <v>61</v>
@@ -3506,7 +3515,7 @@
         <v>27</v>
       </c>
       <c r="K36" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L36" s="5" t="s">
         <v>133</v>
@@ -3532,7 +3541,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C37" s="10" t="s">
         <v>149</v>
@@ -3541,7 +3550,7 @@
         <v>150</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>50</v>
@@ -3559,10 +3568,10 @@
         <v>27</v>
       </c>
       <c r="K37" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L37" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M37" s="10" t="s">
         <v>105</v>
@@ -3585,7 +3594,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>81</v>
@@ -3594,7 +3603,7 @@
         <v>82</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F38" s="5" t="s">
         <v>96</v>
@@ -3612,10 +3621,10 @@
         <v>27</v>
       </c>
       <c r="K38" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M38" s="5" t="s">
         <v>36</v>
@@ -3638,7 +3647,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C39" s="10" t="s">
         <v>117</v>
@@ -3665,10 +3674,10 @@
         <v>27</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="L39" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M39" s="10" t="s">
         <v>58</v>
@@ -3691,7 +3700,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>88</v>
@@ -3700,7 +3709,7 @@
         <v>89</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F40" s="5" t="s">
         <v>127</v>
@@ -3718,7 +3727,7 @@
         <v>27</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L40" s="5" t="s">
         <v>104</v>
@@ -3744,7 +3753,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C41" s="10" t="s">
         <v>20</v>
@@ -3797,7 +3806,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>117</v>
@@ -3824,10 +3833,10 @@
         <v>27</v>
       </c>
       <c r="K42" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M42" s="5" t="s">
         <v>105</v>
@@ -3850,7 +3859,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C43" s="10" t="s">
         <v>149</v>
@@ -3877,7 +3886,7 @@
         <v>27</v>
       </c>
       <c r="K43" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L43" s="10" t="s">
         <v>92</v>
@@ -3903,7 +3912,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>107</v>
@@ -3930,7 +3939,7 @@
         <v>27</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="L44" s="5" t="s">
         <v>127</v>
@@ -3956,7 +3965,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>20</v>
@@ -4009,7 +4018,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>107</v>
@@ -4018,7 +4027,7 @@
         <v>108</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>44</v>
@@ -4036,13 +4045,13 @@
         <v>27</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>152</v>
       </c>
       <c r="M46" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N46" s="5" t="s">
         <v>51</v>
@@ -4062,7 +4071,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C47" s="10" t="s">
         <v>111</v>
@@ -4071,10 +4080,10 @@
         <v>112</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G47" s="10" t="s">
         <v>36</v>
@@ -4089,10 +4098,10 @@
         <v>27</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="L47" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M47" s="10" t="s">
         <v>58</v>
@@ -4115,7 +4124,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>47</v>
@@ -4124,10 +4133,10 @@
         <v>48</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>93</v>
@@ -4142,10 +4151,10 @@
         <v>27</v>
       </c>
       <c r="K48" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M48" s="5" t="s">
         <v>36</v>
@@ -4168,7 +4177,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C49" s="10" t="s">
         <v>54</v>
@@ -4221,7 +4230,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>107</v>
@@ -4248,7 +4257,7 @@
         <v>27</v>
       </c>
       <c r="K50" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L50" s="5" t="s">
         <v>39</v>
@@ -4274,7 +4283,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C51" s="10" t="s">
         <v>47</v>
@@ -4301,7 +4310,7 @@
         <v>27</v>
       </c>
       <c r="K51" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L51" s="10" t="s">
         <v>39</v>
@@ -4327,7 +4336,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>88</v>
@@ -4336,7 +4345,7 @@
         <v>89</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F52" s="5" t="s">
         <v>44</v>
@@ -4354,7 +4363,7 @@
         <v>27</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>130</v>
@@ -4380,7 +4389,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C53" s="10" t="s">
         <v>20</v>
@@ -4433,7 +4442,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C54" s="5" t="s">
         <v>98</v>
@@ -4442,7 +4451,7 @@
         <v>99</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F54" s="5" t="s">
         <v>61</v>
@@ -4460,7 +4469,7 @@
         <v>27</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L54" s="5" t="s">
         <v>39</v>
@@ -4486,7 +4495,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C55" s="10" t="s">
         <v>88</v>
@@ -4495,7 +4504,7 @@
         <v>89</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>92</v>
@@ -4539,7 +4548,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C56" s="5" t="s">
         <v>107</v>
@@ -4548,7 +4557,7 @@
         <v>108</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F56" s="5" t="s">
         <v>35</v>
@@ -4566,7 +4575,7 @@
         <v>27</v>
       </c>
       <c r="K56" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L56" s="5" t="s">
         <v>136</v>
@@ -4592,7 +4601,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C57" s="10" t="s">
         <v>98</v>
@@ -4645,7 +4654,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>20</v>
@@ -4654,7 +4663,7 @@
         <v>21</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F58" s="5" t="s">
         <v>92</v>
@@ -4672,7 +4681,7 @@
         <v>27</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="L58" s="5" t="s">
         <v>61</v>
@@ -4698,7 +4707,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C59" s="10" t="s">
         <v>32</v>
@@ -4707,7 +4716,7 @@
         <v>33</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>50</v>
@@ -4725,10 +4734,10 @@
         <v>27</v>
       </c>
       <c r="K59" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L59" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M59" s="10" t="s">
         <v>58</v>
@@ -4751,7 +4760,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>54</v>
@@ -4804,7 +4813,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C61" s="10" t="s">
         <v>32</v>
@@ -4813,7 +4822,7 @@
         <v>33</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>92</v>
@@ -4857,7 +4866,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>54</v>
@@ -4866,7 +4875,7 @@
         <v>55</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F62" s="5" t="s">
         <v>61</v>
@@ -4875,7 +4884,7 @@
         <v>62</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I62" s="6" t="s">
         <v>26</v>
@@ -4884,7 +4893,7 @@
         <v>27</v>
       </c>
       <c r="K62" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L62" s="5" t="s">
         <v>39</v>
@@ -4910,7 +4919,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C63" s="10" t="s">
         <v>47</v>
@@ -4919,10 +4928,10 @@
         <v>48</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F63" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G63" s="10" t="s">
         <v>93</v>
@@ -4963,7 +4972,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C64" s="5" t="s">
         <v>111</v>
@@ -4972,7 +4981,7 @@
         <v>112</v>
       </c>
       <c r="E64" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F64" s="5" t="s">
         <v>44</v>
@@ -5016,7 +5025,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C65" s="10" t="s">
         <v>81</v>
@@ -5025,13 +5034,13 @@
         <v>82</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>152</v>
       </c>
       <c r="G65" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H65" s="10" t="s">
         <v>51</v>
@@ -5043,10 +5052,10 @@
         <v>27</v>
       </c>
       <c r="K65" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L65" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M65" s="10" t="s">
         <v>93</v>
@@ -5069,7 +5078,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>98</v>
@@ -5078,7 +5087,7 @@
         <v>99</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F66" s="5" t="s">
         <v>127</v>
@@ -5122,7 +5131,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C67" s="10" t="s">
         <v>107</v>
@@ -5175,7 +5184,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C68" s="5" t="s">
         <v>81</v>
@@ -5202,13 +5211,13 @@
         <v>27</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="L68" s="5" t="s">
         <v>152</v>
       </c>
       <c r="M68" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N68" s="5" t="s">
         <v>63</v>
@@ -5228,7 +5237,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C69" s="10" t="s">
         <v>98</v>
@@ -5281,7 +5290,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>111</v>
@@ -5290,10 +5299,10 @@
         <v>112</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F70" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G70" s="5" t="s">
         <v>93</v>
@@ -5308,7 +5317,7 @@
         <v>27</v>
       </c>
       <c r="K70" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L70" s="5" t="s">
         <v>130</v>
@@ -5334,7 +5343,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C71" s="10" t="s">
         <v>65</v>
@@ -5343,7 +5352,7 @@
         <v>66</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>39</v>
@@ -5387,7 +5396,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C72" s="5" t="s">
         <v>20</v>
@@ -5396,10 +5405,10 @@
         <v>21</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G72" s="5" t="s">
         <v>105</v>
@@ -5440,7 +5449,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C73" s="10" t="s">
         <v>98</v>
@@ -5449,13 +5458,13 @@
         <v>99</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>152</v>
       </c>
       <c r="G73" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H73" s="10" t="s">
         <v>51</v>
@@ -5467,7 +5476,7 @@
         <v>27</v>
       </c>
       <c r="K73" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L73" s="10" t="s">
         <v>92</v>
@@ -5493,7 +5502,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C74" s="5" t="s">
         <v>111</v>
@@ -5546,7 +5555,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C75" s="10" t="s">
         <v>98</v>
@@ -5555,7 +5564,7 @@
         <v>99</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>77</v>
@@ -5573,7 +5582,7 @@
         <v>27</v>
       </c>
       <c r="K75" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L75" s="10" t="s">
         <v>104</v>
@@ -5599,7 +5608,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C76" s="5" t="s">
         <v>32</v>
@@ -5626,7 +5635,7 @@
         <v>27</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L76" s="5" t="s">
         <v>23</v>
@@ -5652,7 +5661,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C77" s="10" t="s">
         <v>117</v>
@@ -5661,10 +5670,10 @@
         <v>118</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F77" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G77" s="10" t="s">
         <v>105</v>
@@ -5705,7 +5714,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C78" s="5" t="s">
         <v>111</v>
@@ -5714,10 +5723,10 @@
         <v>112</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F78" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G78" s="5" t="s">
         <v>58</v>
@@ -5732,7 +5741,7 @@
         <v>27</v>
       </c>
       <c r="K78" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="L78" s="5" t="s">
         <v>96</v>
@@ -5758,7 +5767,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C79" s="10" t="s">
         <v>88</v>
@@ -5785,7 +5794,7 @@
         <v>27</v>
       </c>
       <c r="K79" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L79" s="10" t="s">
         <v>92</v>
@@ -5811,7 +5820,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C80" s="5" t="s">
         <v>88</v>
@@ -5838,10 +5847,10 @@
         <v>27</v>
       </c>
       <c r="K80" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L80" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M80" s="5" t="s">
         <v>58</v>
@@ -5864,7 +5873,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C81" s="10" t="s">
         <v>149</v>
@@ -5891,7 +5900,7 @@
         <v>27</v>
       </c>
       <c r="K81" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L81" s="10" t="s">
         <v>74</v>
@@ -5917,7 +5926,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>117</v>
@@ -5926,10 +5935,10 @@
         <v>118</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G82" s="5" t="s">
         <v>93</v>
@@ -5944,7 +5953,7 @@
         <v>27</v>
       </c>
       <c r="K82" s="5" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="L82" s="5" t="s">
         <v>50</v>
@@ -5970,7 +5979,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C83" s="10" t="s">
         <v>98</v>
@@ -5979,7 +5988,7 @@
         <v>99</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>44</v>
@@ -6023,7 +6032,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C84" s="5" t="s">
         <v>81</v>
@@ -6076,7 +6085,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C85" s="10" t="s">
         <v>20</v>
@@ -6085,10 +6094,10 @@
         <v>21</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F85" s="10" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G85" s="10" t="s">
         <v>62</v>
@@ -6129,7 +6138,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C86" s="5" t="s">
         <v>65</v>
@@ -6138,7 +6147,7 @@
         <v>66</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F86" s="5" t="s">
         <v>35</v>
@@ -6156,7 +6165,7 @@
         <v>27</v>
       </c>
       <c r="K86" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="L86" s="5" t="s">
         <v>143</v>
@@ -6182,7 +6191,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C87" s="10" t="s">
         <v>117</v>
@@ -6209,10 +6218,10 @@
         <v>27</v>
       </c>
       <c r="K87" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L87" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M87" s="10" t="s">
         <v>105</v>
@@ -6235,7 +6244,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C88" s="5" t="s">
         <v>65</v>
@@ -6244,7 +6253,7 @@
         <v>66</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F88" s="5" t="s">
         <v>143</v>
@@ -6262,7 +6271,7 @@
         <v>27</v>
       </c>
       <c r="K88" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L88" s="5" t="s">
         <v>23</v>
@@ -6288,7 +6297,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C89" s="10" t="s">
         <v>20</v>
@@ -6341,7 +6350,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C90" s="5" t="s">
         <v>65</v>
@@ -6350,13 +6359,13 @@
         <v>66</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F90" s="5" t="s">
         <v>152</v>
       </c>
       <c r="G90" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H90" s="5" t="s">
         <v>131</v>
@@ -6368,10 +6377,10 @@
         <v>27</v>
       </c>
       <c r="K90" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L90" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="M90" s="5" t="s">
         <v>58</v>
@@ -6394,7 +6403,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C91" s="10" t="s">
         <v>107</v>
@@ -6403,13 +6412,13 @@
         <v>108</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>152</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H91" s="10" t="s">
         <v>51</v>
@@ -6421,7 +6430,7 @@
         <v>27</v>
       </c>
       <c r="K91" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L91" s="10" t="s">
         <v>44</v>
@@ -6447,7 +6456,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C92" s="5" t="s">
         <v>65</v>
@@ -6456,7 +6465,7 @@
         <v>66</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F92" s="5" t="s">
         <v>143</v>
@@ -6500,7 +6509,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C93" s="10" t="s">
         <v>117</v>
@@ -6527,7 +6536,7 @@
         <v>27</v>
       </c>
       <c r="K93" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L93" s="10" t="s">
         <v>44</v>
@@ -6553,7 +6562,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C94" s="5" t="s">
         <v>111</v>
@@ -6580,7 +6589,7 @@
         <v>27</v>
       </c>
       <c r="K94" s="5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L94" s="5" t="s">
         <v>79</v>
@@ -6606,7 +6615,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C95" s="10" t="s">
         <v>54</v>
@@ -6615,7 +6624,7 @@
         <v>55</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>77</v>
@@ -6659,7 +6668,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C96" s="5" t="s">
         <v>47</v>
@@ -6668,10 +6677,10 @@
         <v>48</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F96" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G96" s="5" t="s">
         <v>93</v>
@@ -6712,7 +6721,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C97" s="10" t="s">
         <v>107</v>
@@ -6721,7 +6730,7 @@
         <v>108</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>39</v>
@@ -6739,10 +6748,10 @@
         <v>27</v>
       </c>
       <c r="K97" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="L97" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="M97" s="10" t="s">
         <v>105</v>
@@ -6765,7 +6774,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C98" s="5" t="s">
         <v>98</v>
@@ -6818,7 +6827,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C99" s="10" t="s">
         <v>20</v>
@@ -6827,10 +6836,10 @@
         <v>21</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F99" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G99" s="10" t="s">
         <v>36</v>
@@ -6845,10 +6854,10 @@
         <v>27</v>
       </c>
       <c r="K99" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L99" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="M99" s="10" t="s">
         <v>105</v>
@@ -6871,7 +6880,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C100" s="5" t="s">
         <v>98</v>
@@ -6880,10 +6889,10 @@
         <v>99</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F100" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G100" s="5" t="s">
         <v>58</v>
@@ -6898,10 +6907,10 @@
         <v>27</v>
       </c>
       <c r="K100" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="L100" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M100" s="5" t="s">
         <v>93</v>
@@ -6924,7 +6933,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C101" s="10" t="s">
         <v>117</v>
@@ -6933,10 +6942,10 @@
         <v>118</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F101" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G101" s="10" t="s">
         <v>93</v>
@@ -6951,7 +6960,7 @@
         <v>27</v>
       </c>
       <c r="K101" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L101" s="10" t="s">
         <v>74</v>
@@ -6977,7 +6986,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C102" s="5" t="s">
         <v>107</v>
@@ -6986,7 +6995,7 @@
         <v>108</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F102" s="5" t="s">
         <v>44</v>
@@ -7004,10 +7013,10 @@
         <v>27</v>
       </c>
       <c r="K102" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L102" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M102" s="5" t="s">
         <v>93</v>
@@ -7030,7 +7039,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="10" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C103" s="10" t="s">
         <v>111</v>
@@ -7083,7 +7092,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C104" s="5" t="s">
         <v>81</v>
@@ -7092,13 +7101,13 @@
         <v>82</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F104" s="5" t="s">
         <v>152</v>
       </c>
       <c r="G104" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H104" s="5" t="s">
         <v>131</v>
@@ -7110,10 +7119,10 @@
         <v>27</v>
       </c>
       <c r="K104" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="L104" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M104" s="5" t="s">
         <v>36</v>
@@ -7136,7 +7145,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C105" s="10" t="s">
         <v>111</v>
@@ -7145,7 +7154,7 @@
         <v>112</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>92</v>
@@ -7163,7 +7172,7 @@
         <v>27</v>
       </c>
       <c r="K105" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L105" s="10" t="s">
         <v>39</v>
@@ -7189,7 +7198,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C106" s="5" t="s">
         <v>111</v>
@@ -7242,7 +7251,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C107" s="10" t="s">
         <v>47</v>
@@ -7251,13 +7260,13 @@
         <v>48</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>152</v>
       </c>
       <c r="G107" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H107" s="10" t="s">
         <v>51</v>
@@ -7269,10 +7278,10 @@
         <v>27</v>
       </c>
       <c r="K107" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="L107" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M107" s="10" t="s">
         <v>40</v>
@@ -7295,7 +7304,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C108" s="5" t="s">
         <v>54</v>
@@ -7304,7 +7313,7 @@
         <v>55</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F108" s="5" t="s">
         <v>61</v>
@@ -7348,7 +7357,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C109" s="10" t="s">
         <v>117</v>
@@ -7357,13 +7366,13 @@
         <v>118</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>152</v>
       </c>
       <c r="G109" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H109" s="10" t="s">
         <v>131</v>
@@ -7401,7 +7410,7 @@
         <v>109</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C110" s="5" t="s">
         <v>54</v>
@@ -7428,10 +7437,10 @@
         <v>27</v>
       </c>
       <c r="K110" s="5" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L110" s="5" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="M110" s="5" t="s">
         <v>62</v>
@@ -7454,7 +7463,7 @@
         <v>110</v>
       </c>
       <c r="B111" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C111" s="10" t="s">
         <v>111</v>
@@ -7507,7 +7516,7 @@
         <v>111</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C112" s="5" t="s">
         <v>81</v>
@@ -7516,10 +7525,10 @@
         <v>82</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F112" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G112" s="5" t="s">
         <v>40</v>
@@ -7534,7 +7543,7 @@
         <v>27</v>
       </c>
       <c r="K112" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="L112" s="5" t="s">
         <v>39</v>
@@ -7560,7 +7569,7 @@
         <v>112</v>
       </c>
       <c r="B113" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C113" s="10" t="s">
         <v>88</v>
@@ -7569,7 +7578,7 @@
         <v>89</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F113" s="10" t="s">
         <v>23</v>
@@ -7587,10 +7596,10 @@
         <v>27</v>
       </c>
       <c r="K113" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L113" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M113" s="10" t="s">
         <v>36</v>
@@ -7613,7 +7622,7 @@
         <v>113</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C114" s="5" t="s">
         <v>32</v>
@@ -7622,10 +7631,10 @@
         <v>33</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F114" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G114" s="5" t="s">
         <v>36</v>
@@ -7640,7 +7649,7 @@
         <v>27</v>
       </c>
       <c r="K114" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L114" s="5" t="s">
         <v>136</v>
@@ -7666,7 +7675,7 @@
         <v>114</v>
       </c>
       <c r="B115" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C115" s="10" t="s">
         <v>111</v>
@@ -7719,7 +7728,7 @@
         <v>115</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C116" s="5" t="s">
         <v>65</v>
@@ -7746,7 +7755,7 @@
         <v>27</v>
       </c>
       <c r="K116" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L116" s="5" t="s">
         <v>39</v>
@@ -7772,7 +7781,7 @@
         <v>116</v>
       </c>
       <c r="B117" s="10" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C117" s="10" t="s">
         <v>149</v>
@@ -7781,7 +7790,7 @@
         <v>150</v>
       </c>
       <c r="E117" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F117" s="10" t="s">
         <v>23</v>
@@ -7825,7 +7834,7 @@
         <v>117</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C118" s="5" t="s">
         <v>65</v>
@@ -7834,7 +7843,7 @@
         <v>66</v>
       </c>
       <c r="E118" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F118" s="5" t="s">
         <v>136</v>
@@ -7852,7 +7861,7 @@
         <v>27</v>
       </c>
       <c r="K118" s="5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L118" s="5" t="s">
         <v>104</v>
@@ -7878,7 +7887,7 @@
         <v>118</v>
       </c>
       <c r="B119" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C119" s="10" t="s">
         <v>54</v>
@@ -7887,7 +7896,7 @@
         <v>55</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F119" s="10" t="s">
         <v>61</v>
@@ -7905,7 +7914,7 @@
         <v>27</v>
       </c>
       <c r="K119" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L119" s="10" t="s">
         <v>44</v>
@@ -7931,7 +7940,7 @@
         <v>119</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C120" s="5" t="s">
         <v>88</v>
@@ -7940,7 +7949,7 @@
         <v>89</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F120" s="5" t="s">
         <v>61</v>
@@ -7984,7 +7993,7 @@
         <v>120</v>
       </c>
       <c r="B121" s="10" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C121" s="10" t="s">
         <v>149</v>
@@ -7993,7 +8002,7 @@
         <v>150</v>
       </c>
       <c r="E121" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F121" s="10" t="s">
         <v>35</v>
@@ -8011,7 +8020,7 @@
         <v>27</v>
       </c>
       <c r="K121" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L121" s="10" t="s">
         <v>133</v>
@@ -8037,7 +8046,7 @@
         <v>121</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C122" s="5" t="s">
         <v>88</v>
@@ -8046,7 +8055,7 @@
         <v>89</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F122" s="5" t="s">
         <v>77</v>
@@ -8064,7 +8073,7 @@
         <v>27</v>
       </c>
       <c r="K122" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L122" s="5" t="s">
         <v>130</v>
@@ -8090,7 +8099,7 @@
         <v>122</v>
       </c>
       <c r="B123" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C123" s="10" t="s">
         <v>117</v>
@@ -8117,10 +8126,10 @@
         <v>27</v>
       </c>
       <c r="K123" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L123" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="M123" s="10" t="s">
         <v>62</v>
@@ -8143,7 +8152,7 @@
         <v>123</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C124" s="5" t="s">
         <v>54</v>
@@ -8152,7 +8161,7 @@
         <v>55</v>
       </c>
       <c r="E124" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F124" s="5" t="s">
         <v>61</v>
@@ -8170,10 +8179,10 @@
         <v>27</v>
       </c>
       <c r="K124" s="5" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="L124" s="5" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="M124" s="5" t="s">
         <v>93</v>
@@ -8196,7 +8205,7 @@
         <v>124</v>
       </c>
       <c r="B125" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C125" s="10" t="s">
         <v>107</v>
@@ -8205,7 +8214,7 @@
         <v>108</v>
       </c>
       <c r="E125" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F125" s="10" t="s">
         <v>61</v>
@@ -8223,7 +8232,7 @@
         <v>27</v>
       </c>
       <c r="K125" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="L125" s="10" t="s">
         <v>61</v>
@@ -8249,7 +8258,7 @@
         <v>125</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C126" s="5" t="s">
         <v>107</v>
@@ -8276,7 +8285,7 @@
         <v>27</v>
       </c>
       <c r="K126" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L126" s="5" t="s">
         <v>96</v>
@@ -8302,7 +8311,7 @@
         <v>126</v>
       </c>
       <c r="B127" s="10" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C127" s="10" t="s">
         <v>47</v>
@@ -8311,10 +8320,10 @@
         <v>48</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F127" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G127" s="10" t="s">
         <v>40</v>
@@ -8329,7 +8338,7 @@
         <v>27</v>
       </c>
       <c r="K127" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L127" s="10" t="s">
         <v>39</v>
@@ -8355,7 +8364,7 @@
         <v>127</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C128" s="5" t="s">
         <v>81</v>
@@ -8364,7 +8373,7 @@
         <v>82</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F128" s="5" t="s">
         <v>74</v>
@@ -8382,10 +8391,10 @@
         <v>27</v>
       </c>
       <c r="K128" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="L128" s="5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="M128" s="5" t="s">
         <v>93</v>
@@ -8408,7 +8417,7 @@
         <v>128</v>
       </c>
       <c r="B129" s="10" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C129" s="10" t="s">
         <v>149</v>
@@ -8435,7 +8444,7 @@
         <v>27</v>
       </c>
       <c r="K129" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L129" s="10" t="s">
         <v>92</v>
@@ -8461,7 +8470,7 @@
         <v>129</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C130" s="5" t="s">
         <v>149</v>
@@ -8514,7 +8523,7 @@
         <v>130</v>
       </c>
       <c r="B131" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C131" s="10" t="s">
         <v>88</v>
@@ -8541,7 +8550,7 @@
         <v>27</v>
       </c>
       <c r="K131" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="L131" s="10" t="s">
         <v>104</v>
@@ -8567,7 +8576,7 @@
         <v>131</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C132" s="5" t="s">
         <v>98</v>
@@ -8620,7 +8629,7 @@
         <v>132</v>
       </c>
       <c r="B133" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C133" s="10" t="s">
         <v>81</v>
@@ -8629,7 +8638,7 @@
         <v>82</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F133" s="10" t="s">
         <v>44</v>
@@ -8673,7 +8682,7 @@
         <v>133</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C134" s="5" t="s">
         <v>32</v>
@@ -8682,7 +8691,7 @@
         <v>33</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F134" s="5" t="s">
         <v>61</v>
@@ -8691,7 +8700,7 @@
         <v>62</v>
       </c>
       <c r="H134" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I134" s="6" t="s">
         <v>26</v>
@@ -8700,7 +8709,7 @@
         <v>27</v>
       </c>
       <c r="K134" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L134" s="5" t="s">
         <v>96</v>
@@ -8726,7 +8735,7 @@
         <v>134</v>
       </c>
       <c r="B135" s="10" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C135" s="10" t="s">
         <v>81</v>
@@ -8735,10 +8744,10 @@
         <v>82</v>
       </c>
       <c r="E135" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F135" s="10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G135" s="10" t="s">
         <v>105</v>
@@ -8779,7 +8788,7 @@
         <v>135</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C136" s="5" t="s">
         <v>47</v>
@@ -8788,7 +8797,7 @@
         <v>48</v>
       </c>
       <c r="E136" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F136" s="5" t="s">
         <v>133</v>
@@ -8832,7 +8841,7 @@
         <v>136</v>
       </c>
       <c r="B137" s="10" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C137" s="10" t="s">
         <v>88</v>
@@ -8865,7 +8874,7 @@
         <v>152</v>
       </c>
       <c r="M137" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N137" s="10" t="s">
         <v>51</v>
@@ -8885,7 +8894,7 @@
         <v>137</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C138" s="5" t="s">
         <v>32</v>
@@ -8894,10 +8903,10 @@
         <v>33</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F138" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G138" s="5" t="s">
         <v>40</v>
@@ -8912,13 +8921,13 @@
         <v>27</v>
       </c>
       <c r="K138" s="5" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L138" s="5" t="s">
         <v>152</v>
       </c>
       <c r="M138" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="N138" s="5" t="s">
         <v>131</v>
@@ -8938,7 +8947,7 @@
         <v>138</v>
       </c>
       <c r="B139" s="10" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C139" s="10" t="s">
         <v>65</v>
@@ -8965,7 +8974,7 @@
         <v>27</v>
       </c>
       <c r="K139" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L139" s="10" t="s">
         <v>77</v>
@@ -8991,7 +9000,7 @@
         <v>139</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C140" s="5" t="s">
         <v>149</v>
@@ -9044,7 +9053,7 @@
         <v>140</v>
       </c>
       <c r="B141" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C141" s="10" t="s">
         <v>54</v>
@@ -9053,7 +9062,7 @@
         <v>55</v>
       </c>
       <c r="E141" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F141" s="10" t="s">
         <v>61</v>
@@ -9071,7 +9080,7 @@
         <v>27</v>
       </c>
       <c r="K141" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L141" s="10" t="s">
         <v>44</v>
@@ -9097,7 +9106,7 @@
         <v>141</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C142" s="5" t="s">
         <v>81</v>
@@ -9106,10 +9115,10 @@
         <v>82</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F142" s="5" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G142" s="5" t="s">
         <v>93</v>
@@ -9124,10 +9133,10 @@
         <v>27</v>
       </c>
       <c r="K142" s="5" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="L142" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="M142" s="5" t="s">
         <v>40</v>
@@ -9150,7 +9159,7 @@
         <v>142</v>
       </c>
       <c r="B143" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C143" s="10" t="s">
         <v>32</v>
@@ -9159,7 +9168,7 @@
         <v>33</v>
       </c>
       <c r="E143" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F143" s="10" t="s">
         <v>61</v>
@@ -9168,7 +9177,7 @@
         <v>62</v>
       </c>
       <c r="H143" s="10" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I143" s="11" t="s">
         <v>26</v>
@@ -9177,7 +9186,7 @@
         <v>27</v>
       </c>
       <c r="K143" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L143" s="10" t="s">
         <v>96</v>
@@ -9203,7 +9212,7 @@
         <v>143</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C144" s="5" t="s">
         <v>47</v>
@@ -9212,7 +9221,7 @@
         <v>48</v>
       </c>
       <c r="E144" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F144" s="5" t="s">
         <v>133</v>
@@ -9256,7 +9265,7 @@
         <v>144</v>
       </c>
       <c r="B145" s="10" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C145" s="10" t="s">
         <v>81</v>
@@ -9265,10 +9274,10 @@
         <v>82</v>
       </c>
       <c r="E145" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F145" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G145" s="10" t="s">
         <v>40</v>
@@ -9283,10 +9292,10 @@
         <v>27</v>
       </c>
       <c r="K145" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="L145" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="M145" s="10" t="s">
         <v>93</v>
@@ -9308,17 +9317,17 @@
   <sheetProtection sheet="1" selectLockedCells="1" autoFilter="0"/>
   <autoFilter ref="A1:S145"/>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose A, B, TIE, or INSUFFICIENT_INFO." sqref="Q10:Q145">
-      <formula1>"A,B,TIE,INSUFFICIENT_INFO"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="选择无效" error="请选择 A、B、平局或信息不足。" sqref="Q10:Q145">
+      <formula1>"A,B,平局,信息不足"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid choice" error="Choose A, B, TIE, or INSUFFICIENT_INFO." sqref="Q2:Q145">
-      <formula1>"A,B,TIE,INSUFFICIENT_INFO"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="选择无效" error="请选择 A、B、平局或信息不足。" sqref="Q2:Q145">
+      <formula1>"A,B,平局,信息不足"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid confidence" error="Choose high, medium, or low." sqref="R10:R145">
-      <formula1>"high,medium,low"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="置信度无效" error="请选择高、中或低。" sqref="R10:R145">
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid confidence" error="Choose high, medium, or low." sqref="R2:R145">
-      <formula1>"high,medium,low"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="置信度无效" error="请选择高、中或低。" sqref="R2:R145">
+      <formula1>"高,中,低"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -9915,18 +9924,18 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:2" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="2" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -9934,7 +9943,7 @@
         <v>16</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -9942,55 +9951,55 @@
         <v>17</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -10002,7 +10011,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -10011,31 +10020,31 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:2" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="2" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B4" s="15">
         <v>144</v>
@@ -10043,34 +10052,42 @@
     </row>
     <row r="5" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="6" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="18" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>366</v>
+        <v>367</v>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>369</v>
       </c>
     </row>
   </sheetData>

</xml_diff>